<commit_message>
Final run + lock metrics to fresh output (driver 87% / sub-driver 84%)
- Re-ran the pipeline end to end; refreshed dashboard data and PDFs
- Updated methodology and README to the current numbers

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/cleaned_classified.xlsx
+++ b/outputs/cleaned_classified.xlsx
@@ -917,12 +917,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Brand Perception</t>
+          <t>User Experience</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Thought Leadership</t>
+          <t>Product &amp; Service Quality</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>NFO &amp; Fund Launches</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
@@ -1304,11 +1304,11 @@
         </is>
       </c>
       <c r="AG5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="AG8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
@@ -2480,11 +2480,11 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>SIP Returns &amp; Long-Term Performance</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>Active Asset Allocation &amp; Hybrid Funds</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
@@ -3489,7 +3489,7 @@
         </is>
       </c>
       <c r="AG18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
@@ -3997,11 +3997,11 @@
         </is>
       </c>
       <c r="AG21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>Regulatory, IPO &amp; Corporate Moves</t>
+          <t>Regulatory &amp; IPO Developments</t>
         </is>
       </c>
       <c r="AI21" t="inlineStr">
@@ -4159,7 +4159,7 @@
         </is>
       </c>
       <c r="AG22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
@@ -4323,11 +4323,11 @@
         </is>
       </c>
       <c r="AG23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI23" t="inlineStr">
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="AG27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         </is>
       </c>
       <c r="AG28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI29" t="inlineStr">
@@ -5669,11 +5669,11 @@
         </is>
       </c>
       <c r="AG31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>NFO &amp; Fund Launches</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI31" t="inlineStr">
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="AG32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH32" t="inlineStr">
         <is>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AH34" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI34" t="inlineStr">
@@ -6516,11 +6516,11 @@
         </is>
       </c>
       <c r="AG36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH36" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI36" t="inlineStr">
@@ -6881,7 +6881,7 @@
       </c>
       <c r="AH38" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI38" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="AH39" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>Active Asset Allocation &amp; Hybrid Funds</t>
         </is>
       </c>
       <c r="AI39" t="inlineStr">
@@ -7219,7 +7219,7 @@
         </is>
       </c>
       <c r="AG40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH40" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -8733,11 +8733,11 @@
         </is>
       </c>
       <c r="AG49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>Passive &amp; ETF Investing</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI49" t="inlineStr">
@@ -9397,11 +9397,11 @@
         </is>
       </c>
       <c r="AG53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AH53" t="inlineStr">
         <is>
-          <t>Passive &amp; ETF Investing</t>
+          <t>Active Asset Allocation &amp; Hybrid Funds</t>
         </is>
       </c>
       <c r="AI53" t="inlineStr">
@@ -9563,11 +9563,11 @@
         </is>
       </c>
       <c r="AG54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH54" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI54" t="inlineStr">
@@ -9733,11 +9733,11 @@
         </is>
       </c>
       <c r="AG55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH55" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI55" t="inlineStr">
@@ -9868,7 +9868,7 @@
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="Z56" t="inlineStr">
@@ -9899,11 +9899,11 @@
         </is>
       </c>
       <c r="AG56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH56" t="inlineStr">
         <is>
-          <t>Passive &amp; ETF Investing</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI56" t="inlineStr">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="AH57" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI57" t="inlineStr">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="AH58" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI58" t="inlineStr">
@@ -10571,7 +10571,7 @@
         </is>
       </c>
       <c r="AG60" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH60" t="inlineStr">
         <is>
@@ -10739,7 +10739,7 @@
       </c>
       <c r="AH61" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI61" t="inlineStr">
@@ -11075,11 +11075,11 @@
         </is>
       </c>
       <c r="AG63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH63" t="inlineStr">
         <is>
-          <t>Passive &amp; ETF Investing</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI63" t="inlineStr">
@@ -11241,11 +11241,11 @@
         </is>
       </c>
       <c r="AG64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH64" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI64" t="inlineStr">
@@ -11409,11 +11409,11 @@
         </is>
       </c>
       <c r="AG65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH65" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI65" t="inlineStr">
@@ -11739,7 +11739,7 @@
         </is>
       </c>
       <c r="AG67" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH67" t="inlineStr">
         <is>
@@ -12243,11 +12243,11 @@
         </is>
       </c>
       <c r="AG70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH70" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI70" t="inlineStr">
@@ -12409,11 +12409,11 @@
         </is>
       </c>
       <c r="AG71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH71" t="inlineStr">
         <is>
-          <t>SIP Returns &amp; Long-Term Performance</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI71" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="AH72" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI72" t="inlineStr">
@@ -12915,7 +12915,7 @@
       </c>
       <c r="AH74" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI74" t="inlineStr">
@@ -13083,7 +13083,7 @@
       </c>
       <c r="AH75" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI75" t="inlineStr">
@@ -13747,7 +13747,7 @@
       </c>
       <c r="AH79" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI79" t="inlineStr">
@@ -14349,7 +14349,7 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -14600,11 +14600,11 @@
         </is>
       </c>
       <c r="AG84" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AH84" t="inlineStr">
         <is>
-          <t>NFO &amp; Fund Launches</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI84" t="inlineStr">
@@ -14766,11 +14766,11 @@
         </is>
       </c>
       <c r="AG85" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH85" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI85" t="inlineStr">
@@ -15096,11 +15096,11 @@
         </is>
       </c>
       <c r="AG87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH87" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI87" t="inlineStr">
@@ -15256,7 +15256,7 @@
         </is>
       </c>
       <c r="AG88" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH88" t="inlineStr">
         <is>
@@ -15424,7 +15424,7 @@
       </c>
       <c r="AH89" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI89" t="inlineStr">
@@ -15586,11 +15586,11 @@
         </is>
       </c>
       <c r="AG90" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH90" t="inlineStr">
         <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="AI90" t="inlineStr">
@@ -15847,7 +15847,7 @@
         </is>
       </c>
       <c r="P92" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
@@ -15924,7 +15924,7 @@
         </is>
       </c>
       <c r="AG92" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH92" t="inlineStr">
         <is>
@@ -16088,11 +16088,11 @@
         </is>
       </c>
       <c r="AG93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH93" t="inlineStr">
         <is>
-          <t>SIP Returns &amp; Long-Term Performance</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI93" t="inlineStr">
@@ -16256,11 +16256,11 @@
         </is>
       </c>
       <c r="AG94" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AH94" t="inlineStr">
         <is>
-          <t>NFO &amp; Fund Launches</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="AI94" t="inlineStr">
@@ -16426,7 +16426,7 @@
       </c>
       <c r="AH95" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="AI95" t="inlineStr">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="AG96" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH96" t="inlineStr">
         <is>
@@ -17029,27 +17029,27 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Naren &amp; CIO Market Outlook</t>
+          <t>Passive &amp; ETF Investing</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Statements, interviews, and commentary from S. Naren, Anand Shah, Nimesh Shah, and other ICICI Pru AMC leaders on market direction, sector opportunities, risk warnings, and investment strategy.</t>
+          <t>Discussion of ICICI Prudential's passive fund range — index funds, ETFs, smart-beta, and FoFs — and the broader shift toward passive investing as a core portfolio strategy.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>0.238</v>
+        <v>0.12</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Brand Perception</t>
+          <t>User Experience</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -17060,23 +17060,23 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Passive &amp; ETF Investing</t>
+          <t>SIP Returns &amp; Long-Term Performance</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Discussion of ICICI Pru's passive fund range—index funds, ETFs, smart-beta, and FoFs—including strategy commentary and performance versus active peers.</t>
+          <t>Analysis and rankings of ICICI Prudential funds' historical SIP and lump-sum returns across large-cap, mid-cap, small-cap, hybrid, and multi-asset categories over multi-year horizons.</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E3" t="n">
-        <v>0.316</v>
+        <v>0.409</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17091,23 +17091,23 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NFO &amp; Fund Launches</t>
+          <t>Naren &amp; Leadership Outlook</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Coverage of new fund offerings and scheme launches by ICICI Prudential AMC, including index funds, thematic funds, iSIF long-short funds, and conglomerate-focused equity schemes.</t>
+          <t>Statements, interviews, and market forecasts from ICICI Prudential's senior leaders — especially CIO S. Naren and CEO Nimesh Shah — on equities, sectors, risk, and macro themes.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>0.062</v>
+        <v>0.267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17122,23 +17122,23 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SIP Returns &amp; Long-Term Performance</t>
+          <t>App &amp; Digital Experience</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Articles benchmarking ICICI Prudential funds on SIP wealth creation, NAV milestones, CAGR rankings, and multi-year return comparisons across equity, hybrid, and debt categories.</t>
+          <t>User reviews, complaints, and feedback on the ICICI Prudential MF mobile app covering login failures, UI/UX issues, missing features, and registration problems.</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n">
-        <v>0.267</v>
+        <v>-0.462</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -17147,64 +17147,64 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>App &amp; Digital Experience</t>
+          <t>NFO &amp; Fund Launches</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>User reviews, complaints, and feedback on the ICICI Prudential MF mobile app covering login failures, UI issues, missing features, and registration problems.</t>
+          <t>Coverage of new fund offerings and scheme launches by ICICI Prudential AMC, including iSIF long-short funds, index funds, and thematic/conglomerate equity schemes.</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.462</v>
+        <v>0.083</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>User Experience</t>
+          <t>Brand Perception</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CSR, Events &amp; Financial Literacy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ICICI Prudential AMC's participation in investor education events, CSR initiatives, industry conferences, and financial literacy outreach activities.</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>4</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Active Fund &amp; Portfolio Strategy</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Investor-facing guidance on fund selection across multi-asset, hybrid, large-cap, mid-cap, small-cap, and thematic categories, including expert recommendations and portfolio construction advice.</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>0.5</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>User Experience</t>
+          <t>Brand Perception</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -17215,47 +17215,47 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CSR, Events &amp; Financial Literacy</t>
+          <t>Active Asset Allocation &amp; Hybrid Funds</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ICICI Pru AMC's participation in investor education events, CSR initiatives, industry conferences, and financial literacy outreach including panel discussions and retreats.</t>
+          <t>Debate and guidance on multi-asset, hybrid, and dynamic asset allocation funds, including comparisons of active vs. passive approaches and sector/asset-class rotation views.</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5</v>
+        <v>0.667</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Brand Perception</t>
+          <t>User Experience</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Regulatory, IPO &amp; Corporate Moves</t>
+          <t>Regulatory &amp; IPO Developments</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SEBI approvals, the ICICI Prudential AMC IPO filing, fund closures or grandfathering decisions, GIFT City office inauguration, and other regulatory or corporate developments.</t>
+          <t>SEBI approvals, IPO filings, iSIF regulatory framework, fund restructuring (grandfathering of Passive Multi-Asset FoF), and compliance-related news affecting ICICI Prudential AMC.</t>
         </is>
       </c>
       <c r="D9" t="n">

</xml_diff>